<commit_message>
fix: corregir posicion de datos en plantilla excel de proforma
</commit_message>
<xml_diff>
--- a/storage/plantilla_test.xlsx
+++ b/storage/plantilla_test.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qwe\Documents\personal\senati\projects\practicas\sys_proforma\storage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26534D8D-9B0C-4BD2-9BA3-13E03A977956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D577480-F85D-4FCF-BDE5-1115C39639B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COTIZACION" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">COTIZACION!$3:$7</definedName>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>VENDEDOR:</t>
   </si>
@@ -126,6 +127,18 @@
   </si>
   <si>
     <t>7 DIAS</t>
+  </si>
+  <si>
+    <t>hola</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - dos</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - tres</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - uno cuatro</t>
   </si>
 </sst>
 </file>
@@ -521,6 +534,52 @@
     <xf numFmtId="4" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -542,22 +601,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="17" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -569,40 +616,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3448,6 +3461,76 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1228725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>485775</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="CuadroTexto 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8DE3C23-32F6-C40C-6A52-58176915D771}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5800725" y="1228725"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1100"/>
+            <a:t>hola prueba</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -3752,70 +3835,70 @@
   <sheetData>
     <row r="1" spans="1:10" ht="130.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="49"/>
+      <c r="B3" s="53"/>
       <c r="C3" s="37" t="s">
         <v>15</v>
       </c>
       <c r="D3" s="37"/>
-      <c r="E3" s="51" t="s">
+      <c r="E3" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="49"/>
+      <c r="B4" s="53"/>
       <c r="C4" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="50" t="s">
+      <c r="A5" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="50"/>
+      <c r="B5" s="54"/>
       <c r="C5" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="53" t="s">
+      <c r="E5" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
       <c r="E6" s="5"/>
       <c r="F6" s="12"/>
       <c r="G6" s="5"/>
@@ -3828,10 +3911,10 @@
       <c r="B7" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="55" t="s">
+      <c r="C7" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="56"/>
+      <c r="D7" s="68"/>
       <c r="E7" s="39" t="s">
         <v>22</v>
       </c>
@@ -3850,8 +3933,8 @@
         <v>1</v>
       </c>
       <c r="B8" s="24"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="58"/>
+      <c r="C8" s="69"/>
+      <c r="D8" s="70"/>
       <c r="E8" s="29"/>
       <c r="F8" s="29"/>
       <c r="G8" s="34"/>
@@ -3862,8 +3945,8 @@
         <v>2</v>
       </c>
       <c r="B9" s="24"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="58"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="70"/>
       <c r="E9" s="29"/>
       <c r="F9" s="29"/>
       <c r="G9" s="34"/>
@@ -3875,8 +3958,8 @@
         <v>3</v>
       </c>
       <c r="B10" s="24"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="58"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="70"/>
       <c r="E10" s="29"/>
       <c r="F10" s="29"/>
       <c r="G10" s="34"/>
@@ -3888,8 +3971,8 @@
         <v>4</v>
       </c>
       <c r="B11" s="30"/>
-      <c r="C11" s="59"/>
-      <c r="D11" s="60"/>
+      <c r="C11" s="50"/>
+      <c r="D11" s="51"/>
       <c r="E11" s="29"/>
       <c r="F11" s="29"/>
       <c r="G11" s="23"/>
@@ -3900,8 +3983,8 @@
         <v>5</v>
       </c>
       <c r="B12" s="30"/>
-      <c r="C12" s="59"/>
-      <c r="D12" s="60"/>
+      <c r="C12" s="50"/>
+      <c r="D12" s="51"/>
       <c r="E12" s="29"/>
       <c r="F12" s="29"/>
       <c r="G12" s="23"/>
@@ -3912,8 +3995,8 @@
         <v>6</v>
       </c>
       <c r="B13" s="30"/>
-      <c r="C13" s="59"/>
-      <c r="D13" s="60"/>
+      <c r="C13" s="50"/>
+      <c r="D13" s="51"/>
       <c r="E13" s="29"/>
       <c r="F13" s="29"/>
       <c r="G13" s="23"/>
@@ -3924,8 +4007,8 @@
         <v>7</v>
       </c>
       <c r="B14" s="30"/>
-      <c r="C14" s="59"/>
-      <c r="D14" s="60"/>
+      <c r="C14" s="50"/>
+      <c r="D14" s="51"/>
       <c r="E14" s="29"/>
       <c r="F14" s="29"/>
       <c r="G14" s="23"/>
@@ -3936,8 +4019,8 @@
         <v>8</v>
       </c>
       <c r="B15" s="30"/>
-      <c r="C15" s="59"/>
-      <c r="D15" s="60"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="51"/>
       <c r="E15" s="29"/>
       <c r="F15" s="29"/>
       <c r="G15" s="23"/>
@@ -3948,8 +4031,8 @@
         <v>9</v>
       </c>
       <c r="B16" s="30"/>
-      <c r="C16" s="59"/>
-      <c r="D16" s="60"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="51"/>
       <c r="E16" s="29"/>
       <c r="F16" s="29"/>
       <c r="G16" s="23"/>
@@ -3960,8 +4043,8 @@
         <v>10</v>
       </c>
       <c r="B17" s="30"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="60"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="51"/>
       <c r="E17" s="29"/>
       <c r="F17" s="29"/>
       <c r="G17" s="23"/>
@@ -3972,8 +4055,8 @@
         <v>11</v>
       </c>
       <c r="B18" s="30"/>
-      <c r="C18" s="59"/>
-      <c r="D18" s="60"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="51"/>
       <c r="E18" s="29"/>
       <c r="F18" s="29"/>
       <c r="G18" s="23"/>
@@ -3984,8 +4067,8 @@
         <v>12</v>
       </c>
       <c r="B19" s="30"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="60"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="51"/>
       <c r="E19" s="29"/>
       <c r="F19" s="29"/>
       <c r="G19" s="23"/>
@@ -3996,8 +4079,8 @@
         <v>13</v>
       </c>
       <c r="B20" s="30"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="60"/>
+      <c r="C20" s="50"/>
+      <c r="D20" s="51"/>
       <c r="E20" s="29"/>
       <c r="F20" s="29"/>
       <c r="G20" s="23"/>
@@ -4008,8 +4091,8 @@
         <v>14</v>
       </c>
       <c r="B21" s="30"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="60"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="51"/>
       <c r="E21" s="29"/>
       <c r="F21" s="29"/>
       <c r="G21" s="23"/>
@@ -4020,8 +4103,8 @@
         <v>15</v>
       </c>
       <c r="B22" s="30"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="60"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="51"/>
       <c r="E22" s="29"/>
       <c r="F22" s="29"/>
       <c r="G22" s="23"/>
@@ -4032,8 +4115,8 @@
         <v>16</v>
       </c>
       <c r="B23" s="30"/>
-      <c r="C23" s="59"/>
-      <c r="D23" s="60"/>
+      <c r="C23" s="50"/>
+      <c r="D23" s="51"/>
       <c r="E23" s="29"/>
       <c r="F23" s="29"/>
       <c r="G23" s="23"/>
@@ -4044,8 +4127,8 @@
         <v>17</v>
       </c>
       <c r="B24" s="30"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="60"/>
+      <c r="C24" s="50"/>
+      <c r="D24" s="51"/>
       <c r="E24" s="33"/>
       <c r="F24" s="29"/>
       <c r="G24" s="23"/>
@@ -4056,8 +4139,8 @@
         <v>18</v>
       </c>
       <c r="B25" s="28"/>
-      <c r="C25" s="61"/>
-      <c r="D25" s="62"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="49"/>
       <c r="E25" s="33"/>
       <c r="F25" s="29"/>
       <c r="G25" s="23"/>
@@ -4068,8 +4151,8 @@
         <v>19</v>
       </c>
       <c r="B26" s="28"/>
-      <c r="C26" s="61"/>
-      <c r="D26" s="62"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="49"/>
       <c r="E26" s="33"/>
       <c r="F26" s="29"/>
       <c r="G26" s="23"/>
@@ -4080,8 +4163,8 @@
         <v>20</v>
       </c>
       <c r="B27" s="28"/>
-      <c r="C27" s="61"/>
-      <c r="D27" s="62"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="49"/>
       <c r="E27" s="25"/>
       <c r="F27" s="25"/>
       <c r="G27" s="19"/>
@@ -4092,8 +4175,8 @@
         <v>21</v>
       </c>
       <c r="B28" s="28"/>
-      <c r="C28" s="61"/>
-      <c r="D28" s="62"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="49"/>
       <c r="E28" s="25"/>
       <c r="F28" s="25"/>
       <c r="G28" s="19"/>
@@ -4104,8 +4187,8 @@
         <v>22</v>
       </c>
       <c r="B29" s="28"/>
-      <c r="C29" s="61"/>
-      <c r="D29" s="62"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="49"/>
       <c r="E29" s="25"/>
       <c r="F29" s="25"/>
       <c r="G29" s="19"/>
@@ -4116,8 +4199,8 @@
         <v>23</v>
       </c>
       <c r="B30" s="28"/>
-      <c r="C30" s="61"/>
-      <c r="D30" s="62"/>
+      <c r="C30" s="48"/>
+      <c r="D30" s="49"/>
       <c r="E30" s="25"/>
       <c r="F30" s="25"/>
       <c r="G30" s="19"/>
@@ -4128,8 +4211,8 @@
         <v>24</v>
       </c>
       <c r="B31" s="28"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="62"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="49"/>
       <c r="E31" s="25"/>
       <c r="F31" s="25"/>
       <c r="G31" s="19"/>
@@ -4140,8 +4223,8 @@
         <v>25</v>
       </c>
       <c r="B32" s="28"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="62"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="49"/>
       <c r="E32" s="26"/>
       <c r="F32" s="17"/>
       <c r="G32" s="19"/>
@@ -4152,8 +4235,8 @@
         <v>26</v>
       </c>
       <c r="B33" s="16"/>
-      <c r="C33" s="63"/>
-      <c r="D33" s="64"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="45"/>
       <c r="E33" s="20"/>
       <c r="F33" s="20"/>
       <c r="G33" s="20"/>
@@ -4164,8 +4247,8 @@
         <v>27</v>
       </c>
       <c r="B34" s="16"/>
-      <c r="C34" s="63"/>
-      <c r="D34" s="64"/>
+      <c r="C34" s="44"/>
+      <c r="D34" s="45"/>
       <c r="E34" s="16"/>
       <c r="F34" s="17"/>
       <c r="G34" s="19"/>
@@ -4176,8 +4259,8 @@
         <v>28</v>
       </c>
       <c r="B35" s="31"/>
-      <c r="C35" s="63"/>
-      <c r="D35" s="64"/>
+      <c r="C35" s="44"/>
+      <c r="D35" s="45"/>
       <c r="E35" s="20"/>
       <c r="F35" s="20"/>
       <c r="G35" s="20"/>
@@ -4188,8 +4271,8 @@
         <v>29</v>
       </c>
       <c r="B36" s="31"/>
-      <c r="C36" s="63"/>
-      <c r="D36" s="64"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="45"/>
       <c r="E36" s="20"/>
       <c r="F36" s="20"/>
       <c r="G36" s="20"/>
@@ -4200,8 +4283,8 @@
         <v>30</v>
       </c>
       <c r="B37" s="22"/>
-      <c r="C37" s="65"/>
-      <c r="D37" s="66"/>
+      <c r="C37" s="46"/>
+      <c r="D37" s="47"/>
       <c r="E37" s="20"/>
       <c r="F37" s="20"/>
       <c r="G37" s="20"/>
@@ -4209,11 +4292,11 @@
     </row>
     <row r="38" spans="1:8" s="6" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8"/>
-      <c r="B38" s="42" t="s">
+      <c r="B38" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="C38" s="42"/>
-      <c r="D38" s="42"/>
+      <c r="C38" s="58"/>
+      <c r="D38" s="58"/>
       <c r="E38"/>
       <c r="F38" s="14" t="s">
         <v>3</v>
@@ -4227,11 +4310,11 @@
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="47" t="s">
+      <c r="B39" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="47"/>
-      <c r="D39" s="47"/>
+      <c r="C39" s="63"/>
+      <c r="D39" s="63"/>
       <c r="E39"/>
       <c r="F39" s="35">
         <f>SUM(H8:H19)</f>
@@ -4248,11 +4331,11 @@
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="48" t="s">
+      <c r="B40" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
+      <c r="C40" s="64"/>
+      <c r="D40" s="64"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
@@ -4260,25 +4343,25 @@
     </row>
     <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="69" t="s">
+      <c r="B41" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="C41" s="69"/>
-      <c r="D41" s="68" t="s">
+      <c r="C41" s="65"/>
+      <c r="D41" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="E41" s="45"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="45"/>
+      <c r="E41" s="61"/>
+      <c r="F41" s="61"/>
+      <c r="G41" s="61"/>
+      <c r="H41" s="61"/>
     </row>
     <row r="42" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
-      <c r="B42" s="67" t="s">
+      <c r="B42" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="C42" s="67"/>
-      <c r="D42" s="54" t="s">
+      <c r="C42" s="66"/>
+      <c r="D42" s="42" t="s">
         <v>29</v>
       </c>
       <c r="E42" s="9"/>
@@ -4329,12 +4412,12 @@
       <c r="B47"/>
       <c r="C47"/>
       <c r="D47" s="1"/>
-      <c r="E47" s="46" t="s">
+      <c r="E47" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="F47" s="46"/>
-      <c r="G47" s="46"/>
-      <c r="H47" s="46"/>
+      <c r="F47" s="62"/>
+      <c r="G47" s="62"/>
+      <c r="H47" s="62"/>
     </row>
     <row r="48" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48"/>
@@ -4349,16 +4432,16 @@
       <c r="H48" s="1"/>
     </row>
     <row r="49" spans="1:8" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A49" s="44" t="s">
+      <c r="A49" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="B49" s="44"/>
-      <c r="C49" s="44"/>
-      <c r="D49" s="44"/>
-      <c r="E49" s="44"/>
-      <c r="F49" s="44"/>
-      <c r="G49" s="44"/>
-      <c r="H49" s="44"/>
+      <c r="B49" s="60"/>
+      <c r="C49" s="60"/>
+      <c r="D49" s="60"/>
+      <c r="E49" s="60"/>
+      <c r="F49" s="60"/>
+      <c r="G49" s="60"/>
+      <c r="H49" s="60"/>
     </row>
     <row r="50" spans="1:8" s="6" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="E50" s="4"/>
@@ -4602,37 +4685,6 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="E5:H5"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A49:H49"/>
@@ -4649,6 +4701,37 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C13:D13"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.43307086614173229" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.23622047244094491"/>
@@ -4658,4 +4741,37 @@
   </rowBreaks>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319F0410-3FE8-4622-AD99-79C805753D88}">
+  <dimension ref="B2:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="30.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>